<commit_message>
Stadium Board or Orion Board ka BOM complete ho gaya ha.
</commit_message>
<xml_diff>
--- a/Deliverables/Orion_Board/BOM/Client_BOM.xlsx
+++ b/Deliverables/Orion_Board/BOM/Client_BOM.xlsx
@@ -19,10 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="96">
-  <si>
-    <t>Bill of Material (BOM) for Stadium_Board</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="178">
   <si>
     <t>S. No.</t>
   </si>
@@ -222,9 +219,6 @@
     <t>EEE-HB1E330AP</t>
   </si>
   <si>
-    <t>C4, C10, C13</t>
-  </si>
-  <si>
     <t>C5, C11</t>
   </si>
   <si>
@@ -285,21 +279,12 @@
     <t>R1, R4, R6, R7</t>
   </si>
   <si>
-    <t>Res Thick Film 0805 3.3K Ohm 5% 0.125W</t>
-  </si>
-  <si>
     <t>R2</t>
   </si>
   <si>
-    <t>RC0805JR-073K3L</t>
-  </si>
-  <si>
     <t>±1% 1/8W Thick Film Resistors 150V ±100ppm/℃ -55℃~+155℃ 10kΩ 0805 Chip Resistor - Surface Mount ROHS</t>
   </si>
   <si>
-    <t>R3, R5, R8, R9, R10, R17, R18</t>
-  </si>
-  <si>
     <t>R11, R14</t>
   </si>
   <si>
@@ -307,6 +292,269 @@
   </si>
   <si>
     <t>R13, R16</t>
+  </si>
+  <si>
+    <t>C4, C10, C13, C15, C16, C17, C18, C19</t>
+  </si>
+  <si>
+    <t>SOD323</t>
+  </si>
+  <si>
+    <t>RES SMD 0603 14kOhm 0.1% Paper T/R</t>
+  </si>
+  <si>
+    <t>Res0603</t>
+  </si>
+  <si>
+    <t>RT0603BRE0714KL</t>
+  </si>
+  <si>
+    <t>R3, R5, R8, R9, R10, R17, R18, R19, R20</t>
+  </si>
+  <si>
+    <t>560R</t>
+  </si>
+  <si>
+    <t>14K</t>
+  </si>
+  <si>
+    <t>10K</t>
+  </si>
+  <si>
+    <t>51K</t>
+  </si>
+  <si>
+    <t>715K</t>
+  </si>
+  <si>
+    <t>13K</t>
+  </si>
+  <si>
+    <t>Mosfet</t>
+  </si>
+  <si>
+    <t>Resistor</t>
+  </si>
+  <si>
+    <t>5.1mm 3.5mm Round Button 50mA To 5.1mm SPST 12V SMD Tactile Switche</t>
+  </si>
+  <si>
+    <t>SW1, SW2, SW3, SW4, SW5</t>
+  </si>
+  <si>
+    <t>TS-1187A-C-G-B</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>IC REG LINEAR 5V 500MA SOT223-4</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>UA78M05IDCYR</t>
+  </si>
+  <si>
+    <t>OPTOISOLTR 5KV 4CH TRANS 16-SMD</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>LTV-844S</t>
+  </si>
+  <si>
+    <t>DC5-24V Wireless WIFI LED RGB Controller RGBW Controller IR / RF Remote Control IOS/Android for LED Strip RGB RGBW RGBWW</t>
+  </si>
+  <si>
+    <t>U3</t>
+  </si>
+  <si>
+    <t>ESP8285</t>
+  </si>
+  <si>
+    <t>IC REG BOOST ADJ 2A SOT23-5</t>
+  </si>
+  <si>
+    <t>U4, U5</t>
+  </si>
+  <si>
+    <t>SOT23-5</t>
+  </si>
+  <si>
+    <t>LMR62014XMF/NOPB</t>
+  </si>
+  <si>
+    <t>Switch</t>
+  </si>
+  <si>
+    <t>IC MCU 8BIT 14KB FLASH 28SSOP</t>
+  </si>
+  <si>
+    <t>IC1</t>
+  </si>
+  <si>
+    <t>PIC16F15355-I/SS</t>
+  </si>
+  <si>
+    <t>28SSOP</t>
+  </si>
+  <si>
+    <t>DC Power Receptacle 1.65mm 4.3mm 7A 24V Plugin AC/DC Power Connectors ROHS</t>
+  </si>
+  <si>
+    <t>J1</t>
+  </si>
+  <si>
+    <t>DC-C024E-7A-1.65</t>
+  </si>
+  <si>
+    <t>16 Pin Right angle JST Conn 2 mm Pitch</t>
+  </si>
+  <si>
+    <t>J2</t>
+  </si>
+  <si>
+    <t>0220164-162121</t>
+  </si>
+  <si>
+    <t>CONN HEADER SMD 6POS 2.54MM</t>
+  </si>
+  <si>
+    <t>J3</t>
+  </si>
+  <si>
+    <t>95293-401A06LF</t>
+  </si>
+  <si>
+    <t>Conn Shrouded Header HDR 8 POS 2.54mm Solder RA Thru-Hole SL™ Tube</t>
+  </si>
+  <si>
+    <t>J10</t>
+  </si>
+  <si>
+    <t>0705510042</t>
+  </si>
+  <si>
+    <t>CONN HEADER R/A 6POS 2.54MM</t>
+  </si>
+  <si>
+    <t>J11</t>
+  </si>
+  <si>
+    <t>0705510040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Murata </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TDK </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Darfon </t>
+  </si>
+  <si>
+    <t>---------</t>
+  </si>
+  <si>
+    <t>LCSC</t>
+  </si>
+  <si>
+    <t>Yageo</t>
+  </si>
+  <si>
+    <t>TDK</t>
+  </si>
+  <si>
+    <t>CC0603KRX5R8BB475</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YAGEO </t>
+  </si>
+  <si>
+    <t>ESR25JZPF5600</t>
+  </si>
+  <si>
+    <t>UNI-ROYAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Texas </t>
+  </si>
+  <si>
+    <t>------</t>
+  </si>
+  <si>
+    <t>Aliexpress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bill of Material (BOM) for Orion Board </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panasonic </t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS </t>
+  </si>
+  <si>
+    <t>Mouser</t>
+  </si>
+  <si>
+    <t>--</t>
+  </si>
+  <si>
+    <t>Slkor</t>
+  </si>
+  <si>
+    <t>-----</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diodes </t>
+  </si>
+  <si>
+    <t>---</t>
+  </si>
+  <si>
+    <t>Littelfuse</t>
+  </si>
+  <si>
+    <t>SOT23-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vishay </t>
+  </si>
+  <si>
+    <t>Alibaba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XKB </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOT-223
+</t>
+  </si>
+  <si>
+    <t>Lite-On</t>
+  </si>
+  <si>
+    <t>MagicHome with ESP8285</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Microchip </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amphenol ICC
+</t>
+  </si>
+  <si>
+    <t>Arrow</t>
+  </si>
+  <si>
+    <t>Molex</t>
+  </si>
+  <si>
+    <t>Micro-Semi</t>
   </si>
 </sst>
 </file>
@@ -318,7 +566,7 @@
     <numFmt numFmtId="165" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -407,8 +655,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -427,14 +682,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="28">
+  <borders count="32">
     <border>
       <left/>
       <right/>
@@ -688,17 +937,6 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -790,10 +1028,67 @@
     </border>
     <border>
       <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -808,7 +1103,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="139">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -863,9 +1158,6 @@
     <xf numFmtId="164" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -879,9 +1171,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -914,18 +1203,12 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -937,29 +1220,11 @@
     </xf>
     <xf numFmtId="165" fontId="10" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -968,18 +1233,12 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -989,128 +1248,278 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1388,13 +1797,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S32"/>
+  <dimension ref="A1:S33"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.28515625" customWidth="1"/>
     <col min="3" max="3" width="73" customWidth="1"/>
-    <col min="4" max="4" width="19.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="28.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.7109375" bestFit="1" customWidth="1"/>
@@ -1403,7 +1812,7 @@
     <col min="10" max="10" width="17.42578125" style="6" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="21.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="13.42578125" customWidth="1"/>
     <col min="15" max="15" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="23.42578125" customWidth="1"/>
@@ -1412,944 +1821,1733 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="16.5" thickBot="1">
-      <c r="A1" s="87" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="89"/>
-      <c r="R1" s="90"/>
+      <c r="A1" s="80" t="s">
+        <v>156</v>
+      </c>
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="63"/>
+      <c r="P1" s="63"/>
+      <c r="Q1" s="64"/>
+      <c r="R1" s="65"/>
     </row>
     <row r="2" spans="1:18" ht="16.5" thickBot="1">
       <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="K2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="O2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="P2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="Q2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="R2" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="16.5" thickBot="1">
       <c r="A3" s="2">
         <v>1</v>
       </c>
-      <c r="B3" s="91" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="98" t="s">
-        <v>60</v>
-      </c>
-      <c r="D3" s="9" t="s">
+      <c r="B3" s="66" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="134" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="84" t="s">
+        <v>62</v>
+      </c>
+      <c r="E3" s="85" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" s="85" t="s">
         <v>63</v>
       </c>
-      <c r="E3" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="69" t="s">
-        <v>73</v>
-      </c>
-      <c r="J3" s="94">
+      <c r="G3" s="21" t="s">
+        <v>147</v>
+      </c>
+      <c r="H3" s="21" t="s">
+        <v>145</v>
+      </c>
+      <c r="I3" s="50" t="s">
+        <v>71</v>
+      </c>
+      <c r="J3" s="86">
         <v>2</v>
       </c>
-      <c r="K3" s="23"/>
-      <c r="L3" s="23"/>
-      <c r="M3" s="24"/>
-      <c r="N3" s="25"/>
-      <c r="O3" s="25"/>
-      <c r="P3" s="25"/>
-      <c r="Q3" s="25"/>
-      <c r="R3" s="26"/>
+      <c r="K3" s="40">
+        <f>J3*20</f>
+        <v>40</v>
+      </c>
+      <c r="L3" s="22">
+        <v>20</v>
+      </c>
+      <c r="M3" s="76" t="s">
+        <v>146</v>
+      </c>
+      <c r="N3" s="23">
+        <v>2.6200000000000001E-2</v>
+      </c>
+      <c r="O3" s="23">
+        <f>N3*L3</f>
+        <v>0.52400000000000002</v>
+      </c>
+      <c r="P3" s="23">
+        <v>2.6200000000000001E-2</v>
+      </c>
+      <c r="Q3" s="23">
+        <f>P3*K3</f>
+        <v>1.048</v>
+      </c>
+      <c r="R3" s="24"/>
     </row>
     <row r="4" spans="1:18" ht="16.5" thickBot="1">
       <c r="A4" s="2">
         <v>2</v>
       </c>
-      <c r="B4" s="92"/>
-      <c r="C4" s="98" t="s">
-        <v>61</v>
-      </c>
-      <c r="D4" s="9" t="s">
+      <c r="B4" s="67"/>
+      <c r="C4" s="47" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="72" t="s">
+        <v>64</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="F4" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="E4" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="69" t="s">
+      <c r="G4" s="58" t="s">
+        <v>157</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="I4" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="57">
+        <v>1</v>
+      </c>
+      <c r="K4" s="8">
+        <f t="shared" ref="K4:K31" si="0">J4*20</f>
         <v>20</v>
       </c>
-      <c r="J4" s="94">
-        <v>1</v>
-      </c>
-      <c r="K4" s="8"/>
-      <c r="L4" s="8"/>
-      <c r="M4" s="12"/>
-      <c r="N4" s="17"/>
-      <c r="O4" s="17"/>
-      <c r="P4" s="17"/>
-      <c r="Q4" s="17"/>
-      <c r="R4" s="27"/>
+      <c r="L4" s="8">
+        <v>5</v>
+      </c>
+      <c r="M4" s="81" t="s">
+        <v>158</v>
+      </c>
+      <c r="N4" s="17">
+        <v>0.52</v>
+      </c>
+      <c r="O4" s="17">
+        <f>N4*L4</f>
+        <v>2.6</v>
+      </c>
+      <c r="P4" s="17">
+        <v>0.52</v>
+      </c>
+      <c r="Q4" s="17">
+        <f>P4*K4</f>
+        <v>10.4</v>
+      </c>
+      <c r="R4" s="25"/>
     </row>
-    <row r="5" spans="1:18" ht="16.5" thickBot="1">
+    <row r="5" spans="1:18" ht="26.25" thickBot="1">
       <c r="A5" s="2">
         <v>3</v>
       </c>
-      <c r="B5" s="92"/>
-      <c r="C5" s="98" t="s">
+      <c r="B5" s="67"/>
+      <c r="C5" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="72" t="s">
+        <v>91</v>
+      </c>
+      <c r="E5" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="E5" s="9" t="s">
+      <c r="F5" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F5" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="69" t="s">
-        <v>51</v>
-      </c>
-      <c r="J5" s="94">
+      <c r="G5" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="I5" s="52" t="s">
+        <v>50</v>
+      </c>
+      <c r="J5" s="57">
         <v>3</v>
       </c>
-      <c r="K5" s="8"/>
-      <c r="L5" s="8"/>
-      <c r="M5" s="12"/>
-      <c r="N5" s="17"/>
-      <c r="O5" s="17"/>
-      <c r="P5" s="17"/>
-      <c r="Q5" s="17"/>
-      <c r="R5" s="27"/>
+      <c r="K5" s="8">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+      <c r="L5" s="8">
+        <v>100</v>
+      </c>
+      <c r="M5" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="N5" s="17">
+        <v>5.7999999999999996E-3</v>
+      </c>
+      <c r="O5" s="17">
+        <f>N5*50</f>
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="P5" s="17">
+        <v>5.7999999999999996E-3</v>
+      </c>
+      <c r="Q5" s="17">
+        <f>P5*L5</f>
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="R5" s="25"/>
     </row>
     <row r="6" spans="1:18" ht="16.5" thickBot="1">
       <c r="A6" s="2">
         <v>4</v>
       </c>
-      <c r="B6" s="92"/>
-      <c r="C6" s="98" t="s">
+      <c r="B6" s="67"/>
+      <c r="C6" s="47" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="72" t="s">
+        <v>66</v>
+      </c>
+      <c r="E6" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="E6" s="9" t="s">
+      <c r="F6" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F6" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="69" t="s">
-        <v>52</v>
-      </c>
-      <c r="J6" s="94">
+      <c r="G6" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="I6" s="52" t="s">
+        <v>51</v>
+      </c>
+      <c r="J6" s="57">
         <v>2</v>
       </c>
-      <c r="K6" s="8"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="80"/>
-      <c r="N6" s="17"/>
-      <c r="O6" s="17"/>
-      <c r="P6" s="17"/>
-      <c r="Q6" s="17"/>
-      <c r="R6" s="27"/>
+      <c r="K6" s="8">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="L6" s="7">
+        <v>10</v>
+      </c>
+      <c r="M6" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="N6" s="17">
+        <v>3.6499999999999998E-2</v>
+      </c>
+      <c r="O6" s="17">
+        <f>N6*L6</f>
+        <v>0.36499999999999999</v>
+      </c>
+      <c r="P6" s="17">
+        <v>3.6499999999999998E-2</v>
+      </c>
+      <c r="Q6" s="17">
+        <f>P6*K6</f>
+        <v>1.46</v>
+      </c>
+      <c r="R6" s="25"/>
     </row>
     <row r="7" spans="1:18" s="13" customFormat="1" ht="16.5" thickBot="1">
       <c r="A7" s="2">
         <v>5</v>
       </c>
-      <c r="B7" s="92"/>
-      <c r="C7" s="98" t="s">
+      <c r="B7" s="67"/>
+      <c r="C7" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="72" t="s">
+        <v>67</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="69" t="s">
-        <v>53</v>
-      </c>
-      <c r="J7" s="94">
+      <c r="G7" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="I7" s="52" t="s">
+        <v>52</v>
+      </c>
+      <c r="J7" s="57">
         <v>2</v>
       </c>
-      <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="12"/>
-      <c r="N7" s="17"/>
-      <c r="O7" s="17"/>
-      <c r="P7" s="17"/>
-      <c r="Q7" s="17"/>
-      <c r="R7" s="27"/>
+      <c r="K7" s="8">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="L7" s="8">
+        <v>100</v>
+      </c>
+      <c r="M7" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="N7" s="17">
+        <v>1.6999999999999999E-3</v>
+      </c>
+      <c r="O7" s="17">
+        <f>N7*L7</f>
+        <v>0.16999999999999998</v>
+      </c>
+      <c r="P7" s="17">
+        <v>1.6999999999999999E-3</v>
+      </c>
+      <c r="Q7" s="17">
+        <f>L7*P7</f>
+        <v>0.16999999999999998</v>
+      </c>
+      <c r="R7" s="25"/>
     </row>
     <row r="8" spans="1:18" ht="16.5" thickBot="1">
       <c r="A8" s="2">
         <v>6</v>
       </c>
-      <c r="B8" s="92"/>
-      <c r="C8" s="98" t="s">
+      <c r="B8" s="67"/>
+      <c r="C8" s="47" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="72" t="s">
+        <v>68</v>
+      </c>
+      <c r="E8" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E8" s="9" t="s">
+      <c r="F8" s="77" t="s">
         <v>36</v>
       </c>
-      <c r="F8" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="69" t="s">
-        <v>54</v>
-      </c>
-      <c r="J8" s="94">
+      <c r="G8" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="I8" s="52" t="s">
+        <v>53</v>
+      </c>
+      <c r="J8" s="57">
         <v>2</v>
       </c>
-      <c r="K8" s="30"/>
-      <c r="L8" s="30"/>
-      <c r="M8" s="31"/>
-      <c r="N8" s="32"/>
-      <c r="O8" s="32"/>
-      <c r="P8" s="32"/>
-      <c r="Q8" s="32"/>
-      <c r="R8" s="33"/>
+      <c r="K8" s="8">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="L8" s="43">
+        <v>10</v>
+      </c>
+      <c r="M8" s="53" t="s">
+        <v>146</v>
+      </c>
+      <c r="N8" s="73">
+        <v>5.7000000000000002E-2</v>
+      </c>
+      <c r="O8" s="73">
+        <f>N8*L8</f>
+        <v>0.57000000000000006</v>
+      </c>
+      <c r="P8" s="73">
+        <v>5.7000000000000002E-2</v>
+      </c>
+      <c r="Q8" s="73">
+        <f>P8*K8</f>
+        <v>2.2800000000000002</v>
+      </c>
+      <c r="R8" s="74"/>
     </row>
     <row r="9" spans="1:18" ht="16.5" thickBot="1">
       <c r="A9" s="2">
         <v>7</v>
       </c>
-      <c r="B9" s="93"/>
-      <c r="C9" s="98" t="s">
-        <v>62</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="G9" s="97"/>
-      <c r="H9" s="97"/>
-      <c r="I9" s="99" t="s">
-        <v>51</v>
-      </c>
-      <c r="J9" s="94">
+      <c r="B9" s="68"/>
+      <c r="C9" s="135" t="s">
+        <v>61</v>
+      </c>
+      <c r="D9" s="87" t="s">
+        <v>69</v>
+      </c>
+      <c r="E9" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="G9" s="27" t="s">
+        <v>148</v>
+      </c>
+      <c r="H9" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="I9" s="88" t="s">
+        <v>50</v>
+      </c>
+      <c r="J9" s="89">
         <v>2</v>
       </c>
-      <c r="K9" s="34"/>
-      <c r="L9" s="34"/>
-      <c r="M9" s="35"/>
-      <c r="N9" s="36"/>
-      <c r="O9" s="36"/>
-      <c r="P9" s="36"/>
-      <c r="Q9" s="36"/>
-      <c r="R9" s="61"/>
+      <c r="K9" s="28">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="L9" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="M9" s="90" t="s">
+        <v>159</v>
+      </c>
+      <c r="N9" s="30">
+        <v>0.121</v>
+      </c>
+      <c r="O9" s="30">
+        <f>N9*J9</f>
+        <v>0.24199999999999999</v>
+      </c>
+      <c r="P9" s="30">
+        <v>4.9000000000000002E-2</v>
+      </c>
+      <c r="Q9" s="30">
+        <f>P9*K9</f>
+        <v>1.96</v>
+      </c>
+      <c r="R9" s="31"/>
     </row>
     <row r="10" spans="1:18" ht="16.5" thickBot="1">
       <c r="A10" s="2">
         <v>8</v>
       </c>
-      <c r="B10" s="82" t="s">
-        <v>56</v>
-      </c>
-      <c r="C10" s="98" t="s">
+      <c r="B10" s="59" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" s="134" t="s">
+        <v>72</v>
+      </c>
+      <c r="D10" s="84" t="s">
+        <v>73</v>
+      </c>
+      <c r="E10" s="85" t="s">
         <v>74</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="F10" s="85" t="s">
         <v>75</v>
       </c>
-      <c r="E10" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-      <c r="J10" s="94">
+      <c r="G10" s="21" t="s">
+        <v>161</v>
+      </c>
+      <c r="H10" s="21" t="s">
+        <v>145</v>
+      </c>
+      <c r="I10" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="J10" s="86">
         <v>1</v>
       </c>
-      <c r="K10" s="37"/>
-      <c r="L10" s="37"/>
-      <c r="M10" s="38"/>
-      <c r="N10" s="39"/>
-      <c r="O10" s="39"/>
-      <c r="P10" s="39"/>
-      <c r="Q10" s="39"/>
-      <c r="R10" s="40"/>
+      <c r="K10" s="22">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="L10" s="22">
+        <v>50</v>
+      </c>
+      <c r="M10" s="76" t="s">
+        <v>146</v>
+      </c>
+      <c r="N10" s="23">
+        <v>0.01</v>
+      </c>
+      <c r="O10" s="23">
+        <f>N10*L10</f>
+        <v>0.5</v>
+      </c>
+      <c r="P10" s="23">
+        <v>0.01</v>
+      </c>
+      <c r="Q10" s="23">
+        <f>P10*L10</f>
+        <v>0.5</v>
+      </c>
+      <c r="R10" s="24"/>
     </row>
     <row r="11" spans="1:18" ht="16.5" thickBot="1">
       <c r="A11" s="2">
         <v>9</v>
       </c>
-      <c r="B11" s="84"/>
-      <c r="C11" s="98" t="s">
+      <c r="B11" s="61"/>
+      <c r="C11" s="135" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="87" t="s">
+        <v>76</v>
+      </c>
+      <c r="E11" s="26" t="s">
+        <v>92</v>
+      </c>
+      <c r="F11" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9" t="s">
+      <c r="G11" s="27" t="s">
+        <v>163</v>
+      </c>
+      <c r="H11" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="I11" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="J11" s="89">
+        <v>2</v>
+      </c>
+      <c r="K11" s="28">
+        <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="94">
-        <v>2</v>
-      </c>
-      <c r="K11" s="34"/>
-      <c r="L11" s="34"/>
-      <c r="M11" s="35"/>
-      <c r="N11" s="36"/>
-      <c r="O11" s="36"/>
-      <c r="P11" s="36"/>
-      <c r="Q11" s="36"/>
-      <c r="R11" s="61"/>
+      <c r="L11" s="28">
+        <v>5</v>
+      </c>
+      <c r="M11" s="90" t="s">
+        <v>146</v>
+      </c>
+      <c r="N11" s="30">
+        <v>0.1087</v>
+      </c>
+      <c r="O11" s="30">
+        <f>N11*L11</f>
+        <v>0.54349999999999998</v>
+      </c>
+      <c r="P11" s="30">
+        <v>0.1087</v>
+      </c>
+      <c r="Q11" s="30">
+        <f>P11*K11</f>
+        <v>4.3479999999999999</v>
+      </c>
+      <c r="R11" s="31"/>
     </row>
     <row r="12" spans="1:18" ht="16.5" thickBot="1">
       <c r="A12" s="2">
         <v>10</v>
       </c>
-      <c r="B12" s="70" t="s">
-        <v>82</v>
-      </c>
-      <c r="C12" s="98" t="s">
+      <c r="B12" s="69" t="s">
+        <v>80</v>
+      </c>
+      <c r="C12" s="136" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12" s="95" t="s">
+        <v>78</v>
+      </c>
+      <c r="E12" s="96" t="s">
+        <v>108</v>
+      </c>
+      <c r="F12" s="96" t="s">
         <v>79</v>
       </c>
-      <c r="D12" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="94">
+      <c r="G12" s="97" t="s">
+        <v>165</v>
+      </c>
+      <c r="H12" s="97" t="s">
+        <v>145</v>
+      </c>
+      <c r="I12" s="97" t="s">
+        <v>162</v>
+      </c>
+      <c r="J12" s="98">
         <v>1</v>
       </c>
-      <c r="K12" s="47"/>
-      <c r="L12" s="47"/>
-      <c r="M12" s="48"/>
-      <c r="N12" s="49"/>
-      <c r="O12" s="49"/>
-      <c r="P12" s="49"/>
-      <c r="Q12" s="49"/>
-      <c r="R12" s="50"/>
+      <c r="K12" s="34">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="L12" s="97" t="s">
+        <v>164</v>
+      </c>
+      <c r="M12" s="99" t="s">
+        <v>159</v>
+      </c>
+      <c r="N12" s="35">
+        <v>0.54400000000000004</v>
+      </c>
+      <c r="O12" s="35">
+        <f>N12*J12</f>
+        <v>0.54400000000000004</v>
+      </c>
+      <c r="P12" s="35">
+        <v>0.51200000000000001</v>
+      </c>
+      <c r="Q12" s="35">
+        <f>P12*K12</f>
+        <v>10.24</v>
+      </c>
+      <c r="R12" s="36"/>
     </row>
     <row r="13" spans="1:18" ht="16.5" thickBot="1">
       <c r="A13" s="2">
         <v>11</v>
       </c>
-      <c r="B13" s="70" t="s">
-        <v>83</v>
-      </c>
-      <c r="C13" s="100" t="s">
+      <c r="B13" s="56" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" s="137" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" s="103" t="s">
         <v>41</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="E13" s="104" t="s">
+        <v>108</v>
+      </c>
+      <c r="F13" s="104" t="s">
         <v>42</v>
       </c>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="99" t="s">
-        <v>55</v>
-      </c>
-      <c r="J13" s="94">
+      <c r="G13" s="105" t="s">
+        <v>143</v>
+      </c>
+      <c r="H13" s="105" t="s">
+        <v>145</v>
+      </c>
+      <c r="I13" s="104" t="s">
+        <v>54</v>
+      </c>
+      <c r="J13" s="106">
         <v>1</v>
       </c>
-      <c r="K13" s="23"/>
-      <c r="L13" s="23"/>
-      <c r="M13" s="24"/>
-      <c r="N13" s="25"/>
-      <c r="O13" s="25"/>
-      <c r="P13" s="25"/>
-      <c r="Q13" s="25"/>
-      <c r="R13" s="26"/>
+      <c r="K13" s="107">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="L13" s="107">
+        <v>1</v>
+      </c>
+      <c r="M13" s="108" t="s">
+        <v>146</v>
+      </c>
+      <c r="N13" s="109">
+        <v>0.26910000000000001</v>
+      </c>
+      <c r="O13" s="109">
+        <f>N13*J13</f>
+        <v>0.26910000000000001</v>
+      </c>
+      <c r="P13" s="109">
+        <v>0.20050000000000001</v>
+      </c>
+      <c r="Q13" s="109">
+        <f>P13*K13</f>
+        <v>4.01</v>
+      </c>
+      <c r="R13" s="110"/>
     </row>
     <row r="14" spans="1:18" ht="16.5" thickBot="1">
       <c r="A14" s="2">
         <v>12</v>
       </c>
-      <c r="B14" s="95"/>
-      <c r="C14" s="98" t="s">
+      <c r="B14" s="55" t="s">
+        <v>103</v>
+      </c>
+      <c r="C14" s="138" t="s">
+        <v>82</v>
+      </c>
+      <c r="D14" s="100" t="s">
+        <v>83</v>
+      </c>
+      <c r="E14" s="79" t="s">
+        <v>166</v>
+      </c>
+      <c r="F14" s="79" t="s">
         <v>84</v>
       </c>
-      <c r="D14" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="5">
+      <c r="G14" s="78" t="s">
+        <v>167</v>
+      </c>
+      <c r="H14" s="78" t="s">
+        <v>145</v>
+      </c>
+      <c r="I14" s="78" t="s">
+        <v>162</v>
+      </c>
+      <c r="J14" s="101">
         <v>3</v>
       </c>
-      <c r="K14" s="8"/>
-      <c r="L14" s="8"/>
-      <c r="M14" s="12"/>
-      <c r="N14" s="17"/>
-      <c r="O14" s="17"/>
-      <c r="P14" s="17"/>
-      <c r="Q14" s="17"/>
-      <c r="R14" s="27"/>
+      <c r="K14" s="32">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+      <c r="L14" s="78" t="s">
+        <v>160</v>
+      </c>
+      <c r="M14" s="102" t="s">
+        <v>168</v>
+      </c>
+      <c r="N14" s="33">
+        <v>0.1</v>
+      </c>
+      <c r="O14" s="33">
+        <f>N14*J14</f>
+        <v>0.30000000000000004</v>
+      </c>
+      <c r="P14" s="33">
+        <v>0.1</v>
+      </c>
+      <c r="Q14" s="33">
+        <f>P14*K14</f>
+        <v>6</v>
+      </c>
+      <c r="R14" s="48"/>
     </row>
     <row r="15" spans="1:18" ht="16.5" thickBot="1">
       <c r="A15" s="2">
         <v>13</v>
       </c>
-      <c r="B15" s="95"/>
-      <c r="C15" s="98" t="s">
+      <c r="B15" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="C15" s="134" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="84" t="s">
+        <v>85</v>
+      </c>
+      <c r="E15" s="85" t="s">
         <v>21</v>
       </c>
-      <c r="D15" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="E15" s="9" t="s">
+      <c r="F15" s="91" t="s">
         <v>22</v>
       </c>
-      <c r="F15" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="5">
+      <c r="G15" s="92" t="s">
+        <v>150</v>
+      </c>
+      <c r="H15" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="I15" s="85" t="s">
+        <v>97</v>
+      </c>
+      <c r="J15" s="86">
         <v>4</v>
       </c>
-      <c r="K15" s="8"/>
-      <c r="L15" s="8"/>
-      <c r="M15" s="12"/>
-      <c r="N15" s="17"/>
-      <c r="O15" s="17"/>
-      <c r="P15" s="17"/>
-      <c r="Q15" s="17"/>
-      <c r="R15" s="27"/>
+      <c r="K15" s="22">
+        <f t="shared" si="0"/>
+        <v>80</v>
+      </c>
+      <c r="L15" s="22">
+        <v>10</v>
+      </c>
+      <c r="M15" s="76" t="s">
+        <v>146</v>
+      </c>
+      <c r="N15" s="23">
+        <v>3.4599999999999999E-2</v>
+      </c>
+      <c r="O15" s="23">
+        <f>N15*L15</f>
+        <v>0.34599999999999997</v>
+      </c>
+      <c r="P15" s="23">
+        <v>3.4599999999999999E-2</v>
+      </c>
+      <c r="Q15" s="23">
+        <f>P15*K15</f>
+        <v>2.7679999999999998</v>
+      </c>
+      <c r="R15" s="24"/>
     </row>
     <row r="16" spans="1:18" ht="16.5" thickBot="1">
       <c r="A16" s="2">
         <v>14</v>
       </c>
-      <c r="B16" s="95"/>
-      <c r="C16" s="98" t="s">
-        <v>88</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>89</v>
+      <c r="B16" s="60"/>
+      <c r="C16" s="47" t="s">
+        <v>93</v>
+      </c>
+      <c r="D16" s="72" t="s">
+        <v>86</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>24</v>
+        <v>94</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="G16" s="19"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="5">
+        <v>95</v>
+      </c>
+      <c r="G16" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="H16" s="58" t="s">
+        <v>145</v>
+      </c>
+      <c r="I16" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="J16" s="57">
         <v>1</v>
       </c>
-      <c r="K16" s="8"/>
-      <c r="L16" s="7"/>
-      <c r="M16" s="80"/>
-      <c r="N16" s="17"/>
-      <c r="O16" s="17"/>
-      <c r="P16" s="17"/>
-      <c r="Q16" s="17"/>
-      <c r="R16" s="42"/>
+      <c r="K16" s="8">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="L16" s="7">
+        <v>20</v>
+      </c>
+      <c r="M16" s="53" t="s">
+        <v>146</v>
+      </c>
+      <c r="N16" s="17">
+        <v>2.3800000000000002E-2</v>
+      </c>
+      <c r="O16" s="17">
+        <f>N16*L16</f>
+        <v>0.47600000000000003</v>
+      </c>
+      <c r="P16" s="17">
+        <v>2.3800000000000002E-2</v>
+      </c>
+      <c r="Q16" s="17">
+        <f>P16*K16</f>
+        <v>0.47600000000000003</v>
+      </c>
+      <c r="R16" s="38"/>
     </row>
     <row r="17" spans="1:19" ht="26.25" thickBot="1">
       <c r="A17" s="2">
         <v>15</v>
       </c>
-      <c r="B17" s="95"/>
-      <c r="C17" s="98" t="s">
-        <v>91</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>92</v>
+      <c r="B17" s="60"/>
+      <c r="C17" s="47" t="s">
+        <v>87</v>
+      </c>
+      <c r="D17" s="72" t="s">
+        <v>96</v>
       </c>
       <c r="E17" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F17" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F17" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="G17" s="19"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="5">
-        <v>7</v>
-      </c>
-      <c r="K17" s="8"/>
-      <c r="L17" s="8"/>
-      <c r="M17" s="80"/>
-      <c r="N17" s="17"/>
-      <c r="O17" s="17"/>
-      <c r="P17" s="17"/>
-      <c r="Q17" s="17"/>
-      <c r="R17" s="42"/>
+      <c r="G17" s="58" t="s">
+        <v>152</v>
+      </c>
+      <c r="H17" s="58" t="s">
+        <v>145</v>
+      </c>
+      <c r="I17" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="J17" s="57">
+        <v>9</v>
+      </c>
+      <c r="K17" s="8">
+        <f t="shared" si="0"/>
+        <v>180</v>
+      </c>
+      <c r="L17" s="43">
+        <v>200</v>
+      </c>
+      <c r="M17" s="44" t="s">
+        <v>146</v>
+      </c>
+      <c r="N17" s="17">
+        <v>2.3999999999999998E-3</v>
+      </c>
+      <c r="O17" s="17">
+        <f>N17*100</f>
+        <v>0.24</v>
+      </c>
+      <c r="P17" s="17">
+        <v>2.3999999999999998E-3</v>
+      </c>
+      <c r="Q17" s="17">
+        <f>P17*L17</f>
+        <v>0.48</v>
+      </c>
+      <c r="R17" s="38"/>
     </row>
     <row r="18" spans="1:19" s="11" customFormat="1" ht="15.75" customHeight="1" thickBot="1">
       <c r="A18" s="2">
         <v>16</v>
       </c>
-      <c r="B18" s="96"/>
-      <c r="C18" s="98" t="s">
+      <c r="B18" s="60"/>
+      <c r="C18" s="47" t="s">
+        <v>43</v>
+      </c>
+      <c r="D18" s="72" t="s">
+        <v>88</v>
+      </c>
+      <c r="E18" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="D18" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="E18" s="9" t="s">
+      <c r="F18" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="F18" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="G18" s="29"/>
-      <c r="H18" s="29"/>
-      <c r="I18" s="28"/>
-      <c r="J18" s="5">
+      <c r="G18" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="I18" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="J18" s="57">
         <v>2</v>
       </c>
-      <c r="K18" s="43"/>
-      <c r="L18" s="30"/>
-      <c r="M18" s="44"/>
-      <c r="N18" s="45"/>
-      <c r="O18" s="45"/>
-      <c r="P18" s="45"/>
-      <c r="Q18" s="45"/>
-      <c r="R18" s="46"/>
+      <c r="K18" s="8">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="L18" s="8">
+        <v>100</v>
+      </c>
+      <c r="M18" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="N18" s="15">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="O18" s="17">
+        <f>N18*L18</f>
+        <v>0.11</v>
+      </c>
+      <c r="P18" s="15">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="Q18" s="15">
+        <f>P18*L18</f>
+        <v>0.11</v>
+      </c>
+      <c r="R18" s="93"/>
     </row>
     <row r="19" spans="1:19" s="13" customFormat="1" ht="15.75" customHeight="1" thickBot="1">
       <c r="A19" s="2">
         <v>17</v>
       </c>
-      <c r="B19" s="82" t="s">
-        <v>26</v>
-      </c>
-      <c r="C19" s="98" t="s">
+      <c r="B19" s="60"/>
+      <c r="C19" s="47" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="72" t="s">
+        <v>89</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="F19" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="D19" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="G19" s="41"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
-      <c r="J19" s="5">
+      <c r="G19" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="I19" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="J19" s="57">
         <v>2</v>
       </c>
-      <c r="K19" s="21"/>
-      <c r="L19" s="21"/>
-      <c r="M19" s="81"/>
-      <c r="N19" s="68"/>
-      <c r="O19" s="68"/>
-      <c r="P19" s="68"/>
-      <c r="Q19" s="68"/>
-      <c r="R19" s="62"/>
+      <c r="K19" s="8">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="L19" s="8">
+        <v>100</v>
+      </c>
+      <c r="M19" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="N19" s="17">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="O19" s="17">
+        <f>N19*L19</f>
+        <v>0.12</v>
+      </c>
+      <c r="P19" s="17">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="Q19" s="17">
+        <f>P19*L19</f>
+        <v>0.12</v>
+      </c>
+      <c r="R19" s="25"/>
     </row>
     <row r="20" spans="1:19" ht="16.5" thickBot="1">
       <c r="A20" s="2">
         <v>18</v>
       </c>
-      <c r="B20" s="83"/>
-      <c r="C20" s="98" t="s">
+      <c r="B20" s="61"/>
+      <c r="C20" s="135" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" s="87" t="s">
+        <v>90</v>
+      </c>
+      <c r="E20" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="F20" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="D20" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="G20" s="16"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="5">
+      <c r="G20" s="27" t="s">
+        <v>152</v>
+      </c>
+      <c r="H20" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="I20" s="26" t="s">
+        <v>102</v>
+      </c>
+      <c r="J20" s="89">
         <v>2</v>
       </c>
-      <c r="K20" s="8"/>
-      <c r="L20" s="8"/>
-      <c r="M20" s="14"/>
-      <c r="N20" s="15"/>
-      <c r="O20" s="15"/>
-      <c r="P20" s="15"/>
-      <c r="Q20" s="15"/>
-      <c r="R20" s="58"/>
+      <c r="K20" s="28">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="L20" s="28">
+        <v>100</v>
+      </c>
+      <c r="M20" s="29" t="s">
+        <v>146</v>
+      </c>
+      <c r="N20" s="39">
+        <v>1.5E-3</v>
+      </c>
+      <c r="O20" s="30">
+        <f>N20*L20</f>
+        <v>0.15</v>
+      </c>
+      <c r="P20" s="39">
+        <v>1.5E-3</v>
+      </c>
+      <c r="Q20" s="39">
+        <f>P20*L20</f>
+        <v>0.15</v>
+      </c>
+      <c r="R20" s="94"/>
     </row>
-    <row r="21" spans="1:19" ht="16.5" thickBot="1">
+    <row r="21" spans="1:19" ht="26.25" thickBot="1">
       <c r="A21" s="2">
         <v>19</v>
       </c>
-      <c r="B21" s="83"/>
-      <c r="C21" s="59"/>
-      <c r="D21" s="71"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="16"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="10"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="8"/>
-      <c r="L21" s="8"/>
-      <c r="M21" s="14"/>
-      <c r="N21" s="15"/>
-      <c r="O21" s="15"/>
-      <c r="P21" s="15"/>
-      <c r="Q21" s="15"/>
-      <c r="R21" s="58"/>
+      <c r="B21" s="55" t="s">
+        <v>122</v>
+      </c>
+      <c r="C21" s="138" t="s">
+        <v>105</v>
+      </c>
+      <c r="D21" s="79" t="s">
+        <v>106</v>
+      </c>
+      <c r="E21" s="79" t="s">
+        <v>108</v>
+      </c>
+      <c r="F21" s="79" t="s">
+        <v>107</v>
+      </c>
+      <c r="G21" s="111" t="s">
+        <v>169</v>
+      </c>
+      <c r="H21" s="78" t="s">
+        <v>145</v>
+      </c>
+      <c r="I21" s="78" t="s">
+        <v>154</v>
+      </c>
+      <c r="J21" s="101">
+        <v>5</v>
+      </c>
+      <c r="K21" s="32">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="L21" s="32">
+        <v>10</v>
+      </c>
+      <c r="M21" s="112" t="s">
+        <v>146</v>
+      </c>
+      <c r="N21" s="113">
+        <v>4.8599999999999997E-2</v>
+      </c>
+      <c r="O21" s="33">
+        <f>N21*L21</f>
+        <v>0.48599999999999999</v>
+      </c>
+      <c r="P21" s="113">
+        <v>3.5099999999999999E-2</v>
+      </c>
+      <c r="Q21" s="113">
+        <f>P21*K21</f>
+        <v>3.51</v>
+      </c>
+      <c r="R21" s="133"/>
     </row>
     <row r="22" spans="1:19" ht="16.5" thickBot="1">
       <c r="A22" s="2">
         <v>20</v>
       </c>
-      <c r="B22" s="84"/>
-      <c r="C22" s="60"/>
-      <c r="D22" s="72"/>
-      <c r="E22" s="51"/>
-      <c r="F22" s="51"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="10"/>
-      <c r="I22" s="52"/>
-      <c r="J22" s="53"/>
-      <c r="K22" s="54"/>
-      <c r="L22" s="54"/>
-      <c r="M22" s="55"/>
-      <c r="N22" s="56"/>
-      <c r="O22" s="56"/>
-      <c r="P22" s="56"/>
-      <c r="Q22" s="56"/>
-      <c r="R22" s="63"/>
+      <c r="B22" s="59" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="134" t="s">
+        <v>109</v>
+      </c>
+      <c r="D22" s="85" t="s">
+        <v>110</v>
+      </c>
+      <c r="E22" s="50" t="s">
+        <v>170</v>
+      </c>
+      <c r="F22" s="85" t="s">
+        <v>111</v>
+      </c>
+      <c r="G22" s="114" t="s">
+        <v>153</v>
+      </c>
+      <c r="H22" s="21" t="s">
+        <v>145</v>
+      </c>
+      <c r="I22" s="115" t="s">
+        <v>154</v>
+      </c>
+      <c r="J22" s="116">
+        <v>1</v>
+      </c>
+      <c r="K22" s="22">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="L22" s="22">
+        <v>1</v>
+      </c>
+      <c r="M22" s="117" t="s">
+        <v>146</v>
+      </c>
+      <c r="N22" s="118">
+        <v>1.8105</v>
+      </c>
+      <c r="O22" s="23">
+        <f>N22*L22</f>
+        <v>1.8105</v>
+      </c>
+      <c r="P22" s="118">
+        <v>1.3363</v>
+      </c>
+      <c r="Q22" s="118">
+        <f>P22*K22</f>
+        <v>26.725999999999999</v>
+      </c>
+      <c r="R22" s="119"/>
     </row>
     <row r="23" spans="1:19" s="13" customFormat="1" ht="16.5" thickBot="1">
       <c r="A23" s="2">
         <v>21</v>
       </c>
-      <c r="B23" s="82" t="s">
-        <v>57</v>
-      </c>
-      <c r="C23" s="65"/>
-      <c r="D23" s="73"/>
-      <c r="E23" s="66"/>
-      <c r="F23" s="66"/>
-      <c r="G23" s="57"/>
-      <c r="H23" s="22"/>
-      <c r="I23" s="22"/>
-      <c r="J23" s="57"/>
-      <c r="K23" s="23"/>
-      <c r="L23" s="23"/>
-      <c r="M23" s="24"/>
-      <c r="N23" s="25"/>
-      <c r="O23" s="25"/>
-      <c r="P23" s="25"/>
-      <c r="Q23" s="25"/>
-      <c r="R23" s="67"/>
+      <c r="B23" s="60"/>
+      <c r="C23" s="47" t="s">
+        <v>112</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="G23" s="16" t="s">
+        <v>171</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="I23" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="J23" s="16">
+        <v>1</v>
+      </c>
+      <c r="K23" s="8">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="L23" s="20">
+        <v>10</v>
+      </c>
+      <c r="M23" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="N23" s="51">
+        <v>0.88700000000000001</v>
+      </c>
+      <c r="O23" s="17">
+        <f>N23*L23</f>
+        <v>8.870000000000001</v>
+      </c>
+      <c r="P23" s="51">
+        <v>0.72150000000000003</v>
+      </c>
+      <c r="Q23" s="51">
+        <f>P23*K23</f>
+        <v>14.43</v>
+      </c>
+      <c r="R23" s="75"/>
     </row>
-    <row r="24" spans="1:19" ht="16.5" thickBot="1">
+    <row r="24" spans="1:19" ht="26.25" thickBot="1">
       <c r="A24" s="2">
         <v>22</v>
       </c>
-      <c r="B24" s="83"/>
-      <c r="C24" s="59"/>
-      <c r="D24" s="71"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="16"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="10"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="8"/>
-      <c r="L24" s="8"/>
-      <c r="M24" s="14"/>
-      <c r="N24" s="15"/>
-      <c r="O24" s="15"/>
-      <c r="P24" s="15"/>
-      <c r="Q24" s="15"/>
-      <c r="R24" s="58"/>
+      <c r="B24" s="60"/>
+      <c r="C24" s="47" t="s">
+        <v>115</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="F24" s="41" t="s">
+        <v>172</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="H24" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="I24" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="J24" s="5">
+        <v>1</v>
+      </c>
+      <c r="K24" s="8">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="L24" s="8">
+        <v>20</v>
+      </c>
+      <c r="M24" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="N24" s="15">
+        <v>9.59</v>
+      </c>
+      <c r="O24" s="17">
+        <f>N24*J24</f>
+        <v>9.59</v>
+      </c>
+      <c r="P24" s="15">
+        <v>8.0225000000000009</v>
+      </c>
+      <c r="Q24" s="15">
+        <f>P24*L24</f>
+        <v>160.45000000000002</v>
+      </c>
+      <c r="R24" s="46"/>
     </row>
     <row r="25" spans="1:19" ht="16.5" thickBot="1">
       <c r="A25" s="2">
         <v>23</v>
       </c>
-      <c r="B25" s="83"/>
-      <c r="C25" s="59"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="10"/>
-      <c r="J25" s="5"/>
-      <c r="K25" s="8"/>
-      <c r="L25" s="8"/>
-      <c r="M25" s="14"/>
-      <c r="N25" s="15"/>
-      <c r="O25" s="15"/>
-      <c r="P25" s="15"/>
-      <c r="Q25" s="15"/>
-      <c r="R25" s="58"/>
+      <c r="B25" s="60"/>
+      <c r="C25" s="47" t="s">
+        <v>118</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="G25" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="H25" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="I25" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="J25" s="5">
+        <v>2</v>
+      </c>
+      <c r="K25" s="8">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="L25" s="8">
+        <v>20</v>
+      </c>
+      <c r="M25" s="53" t="s">
+        <v>155</v>
+      </c>
+      <c r="N25" s="17">
+        <v>0.70850000000000002</v>
+      </c>
+      <c r="O25" s="17">
+        <f>N25*L25</f>
+        <v>14.17</v>
+      </c>
+      <c r="P25" s="17">
+        <v>0.53400000000000003</v>
+      </c>
+      <c r="Q25" s="15">
+        <f>P25*K25</f>
+        <v>21.36</v>
+      </c>
+      <c r="R25" s="46"/>
     </row>
     <row r="26" spans="1:19" ht="16.5" thickBot="1">
       <c r="A26" s="2">
         <v>24</v>
       </c>
-      <c r="B26" s="84"/>
-      <c r="C26" s="74"/>
-      <c r="D26" s="75"/>
-      <c r="E26" s="75"/>
-      <c r="F26" s="75"/>
-      <c r="G26" s="76"/>
-      <c r="H26" s="76"/>
-      <c r="I26" s="75"/>
-      <c r="J26" s="77"/>
-      <c r="K26" s="78"/>
-      <c r="L26" s="76"/>
-      <c r="M26" s="76"/>
-      <c r="N26" s="75"/>
-      <c r="O26" s="76"/>
-      <c r="P26" s="76"/>
-      <c r="Q26" s="75"/>
-      <c r="R26" s="79"/>
+      <c r="B26" s="61"/>
+      <c r="C26" s="135" t="s">
+        <v>123</v>
+      </c>
+      <c r="D26" s="26" t="s">
+        <v>124</v>
+      </c>
+      <c r="E26" s="26" t="s">
+        <v>126</v>
+      </c>
+      <c r="F26" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="G26" s="120" t="s">
+        <v>173</v>
+      </c>
+      <c r="H26" s="105" t="s">
+        <v>145</v>
+      </c>
+      <c r="I26" s="121" t="s">
+        <v>154</v>
+      </c>
+      <c r="J26" s="122">
+        <v>1</v>
+      </c>
+      <c r="K26" s="28">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="L26" s="28">
+        <v>1</v>
+      </c>
+      <c r="M26" s="123" t="s">
+        <v>146</v>
+      </c>
+      <c r="N26" s="30">
+        <v>2.7681</v>
+      </c>
+      <c r="O26" s="30">
+        <f>N26*L26</f>
+        <v>2.7681</v>
+      </c>
+      <c r="P26" s="39">
+        <v>2.0196999999999998</v>
+      </c>
+      <c r="Q26" s="39">
+        <f>P26*K26</f>
+        <v>40.393999999999998</v>
+      </c>
+      <c r="R26" s="124"/>
     </row>
     <row r="27" spans="1:19" ht="16.5" thickBot="1">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="G27" s="1"/>
-      <c r="H27" s="1"/>
-      <c r="I27" s="1"/>
-      <c r="J27" s="85" t="s">
-        <v>58</v>
-      </c>
-      <c r="K27" s="85"/>
-      <c r="L27" s="1"/>
-      <c r="M27" s="1"/>
-      <c r="N27" s="1"/>
-      <c r="O27" s="64"/>
-      <c r="P27" s="1"/>
-      <c r="Q27" s="64">
-        <f>SUM(Q3:Q25)</f>
-        <v>0</v>
-      </c>
-      <c r="R27" s="1"/>
-      <c r="S27" s="1"/>
+      <c r="A27" s="2">
+        <v>25</v>
+      </c>
+      <c r="B27" s="59" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" s="134" t="s">
+        <v>127</v>
+      </c>
+      <c r="D27" s="85" t="s">
+        <v>128</v>
+      </c>
+      <c r="E27" s="85" t="s">
+        <v>108</v>
+      </c>
+      <c r="F27" s="85" t="s">
+        <v>129</v>
+      </c>
+      <c r="G27" s="45" t="s">
+        <v>169</v>
+      </c>
+      <c r="H27" s="21" t="s">
+        <v>145</v>
+      </c>
+      <c r="I27" s="115" t="s">
+        <v>154</v>
+      </c>
+      <c r="J27" s="126">
+        <v>1</v>
+      </c>
+      <c r="K27" s="22">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="L27" s="22">
+        <v>1</v>
+      </c>
+      <c r="M27" s="127" t="s">
+        <v>146</v>
+      </c>
+      <c r="N27" s="22">
+        <v>0.74480000000000002</v>
+      </c>
+      <c r="O27" s="22">
+        <f>N27*L27</f>
+        <v>0.74480000000000002</v>
+      </c>
+      <c r="P27" s="118">
+        <v>0.53739999999999999</v>
+      </c>
+      <c r="Q27" s="118">
+        <f>P27*K27</f>
+        <v>10.747999999999999</v>
+      </c>
+      <c r="R27" s="128"/>
     </row>
-    <row r="28" spans="1:19" ht="15.75">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
-      <c r="I28" s="1"/>
-      <c r="J28" s="86" t="s">
-        <v>59</v>
-      </c>
-      <c r="K28" s="86"/>
-      <c r="L28" s="1"/>
-      <c r="M28" s="1"/>
-      <c r="N28" s="1"/>
-      <c r="O28" s="17">
-        <f>SUM(O3:O25)</f>
-        <v>0</v>
-      </c>
-      <c r="P28" s="1"/>
-      <c r="Q28" s="17">
-        <f>Q27/20</f>
-        <v>0</v>
-      </c>
-      <c r="R28" s="1"/>
-      <c r="S28" s="1"/>
+    <row r="28" spans="1:19" ht="16.5" thickBot="1">
+      <c r="A28" s="2">
+        <v>26</v>
+      </c>
+      <c r="B28" s="60"/>
+      <c r="C28" s="47" t="s">
+        <v>130</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="G28" s="37"/>
+      <c r="H28" s="71"/>
+      <c r="I28" s="42" t="s">
+        <v>154</v>
+      </c>
+      <c r="J28" s="5">
+        <v>1</v>
+      </c>
+      <c r="K28" s="8">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="L28" s="8"/>
+      <c r="M28" s="82"/>
+      <c r="N28" s="70"/>
+      <c r="O28" s="17"/>
+      <c r="P28" s="15"/>
+      <c r="Q28" s="15"/>
+      <c r="R28" s="129"/>
     </row>
-    <row r="29" spans="1:19">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
-      <c r="J29" s="1"/>
-      <c r="K29" s="1"/>
-      <c r="L29" s="1"/>
-      <c r="M29" s="1"/>
-      <c r="N29" s="1"/>
-      <c r="O29" s="1"/>
-      <c r="P29" s="1"/>
-      <c r="Q29" s="1"/>
-      <c r="R29" s="1"/>
-      <c r="S29" s="1"/>
+    <row r="29" spans="1:19" ht="16.5" thickBot="1">
+      <c r="A29" s="2">
+        <v>27</v>
+      </c>
+      <c r="B29" s="60"/>
+      <c r="C29" s="47" t="s">
+        <v>133</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="G29" s="37" t="s">
+        <v>174</v>
+      </c>
+      <c r="H29" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="I29" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="J29" s="5">
+        <v>1</v>
+      </c>
+      <c r="K29" s="8">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="L29" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="M29" s="82" t="s">
+        <v>175</v>
+      </c>
+      <c r="N29" s="17">
+        <v>3.15</v>
+      </c>
+      <c r="O29" s="17">
+        <f>N29*J29</f>
+        <v>3.15</v>
+      </c>
+      <c r="P29" s="15">
+        <v>2.7</v>
+      </c>
+      <c r="Q29" s="15">
+        <f>P29*K29</f>
+        <v>54</v>
+      </c>
+      <c r="R29" s="129"/>
     </row>
-    <row r="30" spans="1:19">
-      <c r="A30" s="1"/>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1"/>
-      <c r="K30" s="1"/>
-      <c r="L30" s="1"/>
-      <c r="M30" s="1"/>
-      <c r="N30" s="1"/>
-      <c r="O30" s="1"/>
-      <c r="P30" s="1"/>
-      <c r="Q30" s="1"/>
-      <c r="R30" s="1"/>
+    <row r="30" spans="1:19" ht="16.5" thickBot="1">
+      <c r="A30" s="2">
+        <v>28</v>
+      </c>
+      <c r="B30" s="60"/>
+      <c r="C30" s="47" t="s">
+        <v>136</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="G30" s="37" t="s">
+        <v>176</v>
+      </c>
+      <c r="H30" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="I30" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="J30" s="5">
+        <v>1</v>
+      </c>
+      <c r="K30" s="8">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="L30" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="M30" s="83" t="s">
+        <v>177</v>
+      </c>
+      <c r="N30" s="17">
+        <v>0.877</v>
+      </c>
+      <c r="O30" s="17">
+        <f>N30*J30</f>
+        <v>0.877</v>
+      </c>
+      <c r="P30" s="15">
+        <v>0.79500000000000004</v>
+      </c>
+      <c r="Q30" s="15">
+        <f>P30*K30</f>
+        <v>15.9</v>
+      </c>
+      <c r="R30" s="130"/>
       <c r="S30" s="1"/>
     </row>
-    <row r="31" spans="1:19">
-      <c r="A31" s="1"/>
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
-      <c r="J31" s="1"/>
-      <c r="K31" s="1"/>
-      <c r="L31" s="1"/>
-      <c r="M31" s="1"/>
-      <c r="N31" s="1"/>
-      <c r="O31" s="1"/>
-      <c r="P31" s="1"/>
-      <c r="Q31" s="1"/>
-      <c r="R31" s="1"/>
+    <row r="31" spans="1:19" ht="16.5" thickBot="1">
+      <c r="A31" s="2">
+        <v>29</v>
+      </c>
+      <c r="B31" s="61"/>
+      <c r="C31" s="135" t="s">
+        <v>139</v>
+      </c>
+      <c r="D31" s="26" t="s">
+        <v>140</v>
+      </c>
+      <c r="E31" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="F31" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="G31" s="120" t="s">
+        <v>176</v>
+      </c>
+      <c r="H31" s="105" t="s">
+        <v>145</v>
+      </c>
+      <c r="I31" s="121" t="s">
+        <v>154</v>
+      </c>
+      <c r="J31" s="122">
+        <v>1</v>
+      </c>
+      <c r="K31" s="28">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="L31" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="M31" s="131" t="s">
+        <v>177</v>
+      </c>
+      <c r="N31" s="30">
+        <v>0.72099999999999997</v>
+      </c>
+      <c r="O31" s="30">
+        <f>N31*J31</f>
+        <v>0.72099999999999997</v>
+      </c>
+      <c r="P31" s="39">
+        <v>0.65500000000000003</v>
+      </c>
+      <c r="Q31" s="39">
+        <f>P31*K31</f>
+        <v>13.100000000000001</v>
+      </c>
+      <c r="R31" s="132"/>
       <c r="S31" s="1"/>
     </row>
-    <row r="32" spans="1:19">
+    <row r="32" spans="1:19" ht="16.5" thickBot="1">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
-      <c r="I32" s="1"/>
-      <c r="J32" s="1"/>
-      <c r="K32" s="1"/>
+      <c r="J32" s="125" t="s">
+        <v>57</v>
+      </c>
+      <c r="K32" s="125"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
       <c r="N32" s="1"/>
-      <c r="O32" s="1"/>
+      <c r="O32" s="49"/>
       <c r="P32" s="1"/>
-      <c r="Q32" s="1"/>
+      <c r="Q32" s="49">
+        <f>SUM(Q3:Q31)</f>
+        <v>407.71800000000002</v>
+      </c>
       <c r="R32" s="1"/>
       <c r="S32" s="1"/>
     </row>
+    <row r="33" spans="10:17" ht="15.75">
+      <c r="J33" s="62" t="s">
+        <v>58</v>
+      </c>
+      <c r="K33" s="62"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="17">
+        <f>SUM(O3:O32)</f>
+        <v>51.54699999999999</v>
+      </c>
+      <c r="P33" s="1"/>
+      <c r="Q33" s="17">
+        <f>Q32/20</f>
+        <v>20.385899999999999</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="B23:B26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
+  <mergeCells count="8">
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="J33:K33"/>
     <mergeCell ref="A1:R1"/>
-    <mergeCell ref="B19:B22"/>
     <mergeCell ref="B3:B9"/>
     <mergeCell ref="B10:B11"/>
+    <mergeCell ref="B15:B20"/>
+    <mergeCell ref="B27:B31"/>
+    <mergeCell ref="B22:B26"/>
   </mergeCells>
   <conditionalFormatting sqref="O3:O15">
-    <cfRule type="dataBar" priority="15">
+    <cfRule type="dataBar" priority="22">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -2363,7 +3561,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q3:Q15">
-    <cfRule type="dataBar" priority="13">
+    <cfRule type="dataBar" priority="20">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -2376,8 +3574,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J3:K3 J4:J17 K4:K26">
-    <cfRule type="colorScale" priority="20">
+  <conditionalFormatting sqref="J3:K3 J4:J17 K4:K31">
+    <cfRule type="colorScale" priority="27">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -2388,8 +3586,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J18:J26">
-    <cfRule type="colorScale" priority="10">
+  <conditionalFormatting sqref="J18:J25">
+    <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -2401,7 +3599,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O16">
-    <cfRule type="dataBar" priority="9">
+    <cfRule type="dataBar" priority="16">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -2415,7 +3613,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q16">
-    <cfRule type="dataBar" priority="8">
+    <cfRule type="dataBar" priority="15">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -2429,7 +3627,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O17">
-    <cfRule type="dataBar" priority="7">
+    <cfRule type="dataBar" priority="14">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -2443,7 +3641,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q17">
-    <cfRule type="dataBar" priority="6">
+    <cfRule type="dataBar" priority="13">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -2457,7 +3655,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R18">
-    <cfRule type="dataBar" priority="26">
+    <cfRule type="dataBar" priority="33">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -2471,7 +3669,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R19">
-    <cfRule type="dataBar" priority="27">
+    <cfRule type="dataBar" priority="34">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -2484,8 +3682,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O27">
-    <cfRule type="dataBar" priority="5">
+  <conditionalFormatting sqref="O32">
+    <cfRule type="dataBar" priority="12">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -2498,8 +3696,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q27">
-    <cfRule type="dataBar" priority="4">
+  <conditionalFormatting sqref="Q32">
+    <cfRule type="dataBar" priority="11">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -2512,8 +3710,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q28">
-    <cfRule type="dataBar" priority="2">
+  <conditionalFormatting sqref="Q33">
+    <cfRule type="dataBar" priority="9">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -2526,7 +3724,61 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O28">
+  <conditionalFormatting sqref="J26:J31">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O18:O26 O28:O29">
+    <cfRule type="dataBar" priority="4">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{1BFDD91B-D11F-4318-910D-81019E4B31A6}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O30">
+    <cfRule type="dataBar" priority="3">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{9EA755F1-C025-4D58-94E6-65359B37CDA3}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O31">
+    <cfRule type="dataBar" priority="2">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{2350DDB0-C313-4FE9-ADFC-030A7019B7EF}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O33">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="min"/>
@@ -2535,13 +3787,42 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DA4ECA4C-0B65-46F0-A3F5-6C8C57AE6F27}</x14:id>
+          <x14:id>{EBD71BC8-AE95-42CA-A15F-2F27758F8889}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink ref="M5" r:id="rId1"/>
+    <hyperlink ref="M6" r:id="rId2"/>
+    <hyperlink ref="M7" r:id="rId3"/>
+    <hyperlink ref="M3" r:id="rId4"/>
+    <hyperlink ref="M8" r:id="rId5"/>
+    <hyperlink ref="M15" r:id="rId6"/>
+    <hyperlink ref="M17" r:id="rId7"/>
+    <hyperlink ref="M18" r:id="rId8"/>
+    <hyperlink ref="M19" r:id="rId9"/>
+    <hyperlink ref="M20" r:id="rId10"/>
+    <hyperlink ref="M25" r:id="rId11"/>
+    <hyperlink ref="M4" r:id="rId12"/>
+    <hyperlink ref="M9" r:id="rId13"/>
+    <hyperlink ref="M10" r:id="rId14"/>
+    <hyperlink ref="M11" r:id="rId15"/>
+    <hyperlink ref="M12" r:id="rId16"/>
+    <hyperlink ref="M14" r:id="rId17"/>
+    <hyperlink ref="M16" r:id="rId18"/>
+    <hyperlink ref="M21" r:id="rId19"/>
+    <hyperlink ref="M22" r:id="rId20"/>
+    <hyperlink ref="M23" r:id="rId21"/>
+    <hyperlink ref="M24" r:id="rId22"/>
+    <hyperlink ref="M26" r:id="rId23"/>
+    <hyperlink ref="M27" r:id="rId24"/>
+    <hyperlink ref="M29" r:id="rId25"/>
+    <hyperlink ref="M30" r:id="rId26"/>
+    <hyperlink ref="M31" r:id="rId27"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId28"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -2660,7 +3941,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>O27</xm:sqref>
+          <xm:sqref>O32</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{B2B3B4A6-4811-4007-BF5E-106E1DFA73B6}">
@@ -2673,7 +3954,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>Q27</xm:sqref>
+          <xm:sqref>Q32</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{F97E9DBD-6126-466E-829A-BB8AB2C09E99}">
@@ -2686,10 +3967,49 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>Q28</xm:sqref>
+          <xm:sqref>Q33</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DA4ECA4C-0B65-46F0-A3F5-6C8C57AE6F27}">
+          <x14:cfRule type="dataBar" id="{1BFDD91B-D11F-4318-910D-81019E4B31A6}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>O18:O26 O28:O29</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{9EA755F1-C025-4D58-94E6-65359B37CDA3}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>O30</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{2350DDB0-C313-4FE9-ADFC-030A7019B7EF}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>O31</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{EBD71BC8-AE95-42CA-A15F-2F27758F8889}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -2699,7 +4019,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>O28</xm:sqref>
+          <xm:sqref>O33</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>